<commit_message>
Ground truths need to be updated for GT 3 and 4
Ground truths from pooling were not incorporated into excel files 3 and 4 after judge review.

This had a significant impact ot the RRF script results.

Before and after updating GT:
Done. Here's the comparison with the pooling GT doc_ids now included:

Type	Before Update	After Update	Change
Type 1	100.0%	100.0%	—
Type 2	100.0%	100.0%	—
Type 3	20.7% (18/87)	46.5% (60/129)	+42 new expected docs, found 42 more
Type 4	27.0% (20/74)	60.9% (84/138)	+64 new expected docs, found 64 more
Type 5	79.9%	79.9%	—
Type 6	9.4%	9.4%	—
The pooling GT additions made a big impact:

Type 3 recall jumped from 20.7% → 46.5%, median rank improved from 80 → 24
Type 4 recall jumped from 27.0% → 60.9%, median rank improved from 13 → 46
The ~Gt docs from the judge review are being found by the retrieval system much more effectively than the original expected docs, which makes sense — they were discovered through the retrieval system during pooling
</commit_message>
<xml_diff>
--- a/data/potential_queries/queries_type_3.xlsx
+++ b/data/potential_queries/queries_type_3.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Queries" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,42 +415,34 @@
   </sheetPr>
   <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>query_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>query_type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>query_texts</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>expected_doc_ids</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>filter_criteria</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -472,10 +454,8 @@
           <t>Q3_001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B2" t="n">
+        <v>3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -484,7 +464,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>["NK-ntNa6xcjdwGRXzxV6wpxfd", "NK-cfWFCgJ7etMfnZSJx4xSsb", "NK-GFtNiBqrmJG8ofBNQt97hF", "NK-Wv2e4rkvjjKptipYph5nv7", "NK-SCWNRatvQgpQFUnd8zS4A7", "NK-irZCKsygfBbdat8u2JB7ui", "NK-cxdpQ8HhWX9XXLq9zVonUB", "NK-UN2ZMUxjk6ZYNP5bqyUUxe", "NK-FoHPKahRH6oYTxbT7Tycjk", "NK-AJdA3Gt5CuYSxKVuUAfQfy"]</t>
+          <t>["NK-ntNa6xcjdwGRXzxV6wpxfd", "NK-cfWFCgJ7etMfnZSJx4xSsb", "NK-GFtNiBqrmJG8ofBNQt97hF", "NK-Wv2e4rkvjjKptipYph5nv7", "NK-SCWNRatvQgpQFUnd8zS4A7", "NK-irZCKsygfBbdat8u2JB7ui", "NK-cxdpQ8HhWX9XXLq9zVonUB", "NK-UN2ZMUxjk6ZYNP5bqyUUxe", "NK-FoHPKahRH6oYTxbT7Tycjk", "NK-AJdA3Gt5CuYSxKVuUAfQfy", "NK-3YpnvEwEcL9Jiy7j7tR7nT", "NK-65Ua8srUYwCrD4v89EF5W7", "NK-7RkwYW7dKkaNfppk8DfEka", "NK-F4rVsVTHVMVF4PCwS5WCUP", "NK-GP4PxTt8GsMYQ3Lf3YFWpL", "NK-HG7zmFbtvFquLYgyK9Zuhv", "NK-HoHtMLF9BQuRJmAdicR4cQ", "NK-LSqLFHSaEm45HMAAAtyWHm", "NK-LTtczqzSyDLFwNDam9VpUY", "NK-PQcBwEZ3uBzh34tAGGUpmv", "NK-RyknxxFqBwtgmatsj6s9P8", "NK-WiJhLLmMrT8CFbnJmZHNHk", "NK-X3nYCegg8VTorFeSCceWPX", "NK-Xo4kJnVytBbbXPzeySj98m", "NK-Y4DzsPR3HDoTiFgDDYM42E", "NK-g5CnNukVAMXzCsrG9UpTY8", "NK-gGz7BbryCSo4JZSujy7XFt", "NK-hCyznYUB5a5L75gDVb376t", "NK-kKmdPdAXaFCdqrJfubLxjZ", "NK-nSyzRM3B5eneEE7H2qUQhp", "ua-ws-vessel-1194", "ua-ws-vessel-1209", "ua-ws-vessel-1302", "ua-ws-vessel-1303", "ua-ws-vessel-1334", "ua-ws-vessel-1464", "ua-ws-vessel-1481", "ua-ws-vessel-1486", "ua-ws-vessel-902"]</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -500,10 +480,8 @@
           <t>Q3_002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B3" t="n">
+        <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -512,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>["NK-MYHWYA7zLoQoGrPfVPUcYt", "NK-MVtCt6RAzxf245XiueFWJp", "NK-EQ3dGe5XJhvdMYtQfvKVsP", "kprusi-6bf4f6bf84f9b42a737a9bdf27e84bae9f396585", "NK-Xv8CnM8sgddxx7QenotGtb"]</t>
+          <t>["NK-MYHWYA7zLoQoGrPfVPUcYt", "NK-MVtCt6RAzxf245XiueFWJp", "NK-EQ3dGe5XJhvdMYtQfvKVsP", "kprusi-6bf4f6bf84f9b42a737a9bdf27e84bae9f396585", "NK-Xv8CnM8sgddxx7QenotGtb", "NK-C6kVdiZt3ViKj7rNCHoCyL"]</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -528,10 +506,8 @@
           <t>Q3_003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B4" t="n">
+        <v>3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -540,7 +516,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>["NK-fjaabCsg83J67wd2T3LXoP", "NK-EL5cFqL5pRrFRBSUjny38g", "NK-FoHPKahRH6oYTxbT7Tycjk", "NK-AJdA3Gt5CuYSxKVuUAfQfy"]</t>
+          <t>["NK-fjaabCsg83J67wd2T3LXoP", "NK-EL5cFqL5pRrFRBSUjny38g", "NK-FoHPKahRH6oYTxbT7Tycjk", "NK-AJdA3Gt5CuYSxKVuUAfQfy", "NK-AHmLBXShgacRH3Doimkdv7", "NK-EgaDHFsaqRWDPrZHnNGvnC", "NK-L2aciRRmEVreWptGzTA5MQ", "NK-RNLrSTsR2ixTEVWMeJprzC", "NK-T99fVT6rNS6tGYTK3mRfGN", "NK-ZPgio3iF8qCHLyExLUeauX", "NK-bCjPZb28YG549GoacB5PvD", "NK-euCcvPeH3UduiJAFhgdYQh", "NK-hL3Xv56XN3YqB5QYVcCa22", "NK-hyKMzKozPsV2LaNZtDqqoC"]</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -556,10 +532,8 @@
           <t>Q3_004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B5" t="n">
+        <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -584,10 +558,8 @@
           <t>Q3_005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B6" t="n">
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -612,10 +584,8 @@
           <t>Q3_006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B7" t="n">
+        <v>3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -640,10 +610,8 @@
           <t>Q3_007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B8" t="n">
+        <v>3</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -668,10 +636,8 @@
           <t>Q3_008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B9" t="n">
+        <v>3</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -696,10 +662,8 @@
           <t>Q3_009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B10" t="n">
+        <v>3</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -724,10 +688,8 @@
           <t>Q3_010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B11" t="n">
+        <v>3</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -752,10 +714,8 @@
           <t>Q3_011</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B12" t="n">
+        <v>3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -780,10 +740,8 @@
           <t>Q3_012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B13" t="n">
+        <v>3</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -808,10 +766,8 @@
           <t>Q3_013</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B14" t="n">
+        <v>3</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -820,7 +776,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>["Q461631", "NK-Nz46UHrXiSCEWLkEQTdoPb", "NK-jF6xZDZzsiGDtJtGcBqoLi"]</t>
+          <t>["Q461631", "NK-Nz46UHrXiSCEWLkEQTdoPb", "NK-jF6xZDZzsiGDtJtGcBqoLi", "NK-ZX5STsrwmWoMYSEzL2iQ57"]</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -836,10 +792,8 @@
           <t>Q3_014</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B15" t="n">
+        <v>3</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -848,7 +802,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>["NK-Xv8CnM8sgddxx7QenotGtb", "fbi-lazarus-2876490857c62ddcf8bf089eebd691ed739074dc", "fbi-lazarus-16600ec2ce87bbe1d621bc8a49126cdbd941ae80", "fbi-lazarus-3d52db0cd5be811f997a3c478bc7548690ed85a2", "fbi-lazarus-190b60b8a64fdc41c4468b99f47750d611523ae8", "fbi-lazarus-361c34aeea7771f0c4ae91d97f8769b07d6931c3", "fbi-lazarus-240bb5407be646f7f768d35f0ceb547945d96c8d", "fbi-lazarus-4f05d698ddad088da2e2ce2bf93b6073c93241c5", "fbi-lazarus-55e66b1975218a062a36f86b3d2483c82c265742", "fbi-lazarus-204f6c38bd61b2bda3c864a7eccbf7b0a14f8e57", "fbi-lazarus-19b06e8cd602f407780c2abf2ae1099e70adcdcf"]</t>
+          <t>["NK-Xv8CnM8sgddxx7QenotGtb", "fbi-lazarus-2876490857c62ddcf8bf089eebd691ed739074dc", "fbi-lazarus-16600ec2ce87bbe1d621bc8a49126cdbd941ae80", "fbi-lazarus-3d52db0cd5be811f997a3c478bc7548690ed85a2", "fbi-lazarus-190b60b8a64fdc41c4468b99f47750d611523ae8", "fbi-lazarus-361c34aeea7771f0c4ae91d97f8769b07d6931c3", "fbi-lazarus-240bb5407be646f7f768d35f0ceb547945d96c8d", "fbi-lazarus-4f05d698ddad088da2e2ce2bf93b6073c93241c5", "fbi-lazarus-55e66b1975218a062a36f86b3d2483c82c265742", "fbi-lazarus-204f6c38bd61b2bda3c864a7eccbf7b0a14f8e57", "fbi-lazarus-19b06e8cd602f407780c2abf2ae1099e70adcdcf", "NK-EQ3dGe5XJhvdMYtQfvKVsP"]</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -864,10 +818,8 @@
           <t>Q3_015</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B16" t="n">
+        <v>3</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -892,10 +844,8 @@
           <t>Q3_016</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B17" t="n">
+        <v>3</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -920,10 +870,8 @@
           <t>Q3_017</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B18" t="n">
+        <v>3</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -948,10 +896,8 @@
           <t>Q3_018</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B19" t="n">
+        <v>3</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>

</xml_diff>